<commit_message>
Inventory templates v2: batch/lot + storage location, Replaces Inventory Item, Available Today, clearer units + Hanson notes
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventory-templates/Bean-Avenue-Inventory-Templates.xlsx
+++ b/inventory-templates/Bean-Avenue-Inventory-Templates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9a20525761c98d90/Desktop/Bean Project/Bean_Avenue/inventory-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{5CBE7DA1-B6A9-40A3-96CC-41E50D8D86C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17A6006D-3E19-4F72-9D08-2BF28FD616E0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1619C306-A989-4B43-8B07-B74329623863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="18432" windowHeight="10680" xr2:uid="{7C2AD3C7-4758-4B73-B7C1-F9EA5BA101BC}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="18432" windowHeight="10680" xr2:uid="{01853C2F-0CD5-48E7-83C3-80B3D9719D3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="2" r:id="rId1"/>
@@ -43,33 +43,42 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="114">
-  <si>
-    <t>Bean Avenue - Inventory Import Templates</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="136">
+  <si>
+    <t>Topic</t>
+  </si>
+  <si>
+    <t>Explanation</t>
   </si>
   <si>
     <t>HOW TO USE</t>
   </si>
   <si>
-    <t>Fill the 4 tabs, then import them in Admin &gt; Inventory &gt; Import (one tab at a time or the whole workbook).</t>
-  </si>
-  <si>
-    <t>UNITS - IMPORTANT</t>
-  </si>
-  <si>
-    <t>Always use BASE units: g (grams), ml (millilitres), pc (pieces). Do NOT use kg or litres - the system does not auto-convert. Enter 5000 g, not 5 kg. Enter 20000 ml, not 20 L.</t>
+    <t>Fill the 4 tabs, then import them in Admin &gt; Inventory &gt; Import (one tab at a time or the whole workbook). Nothing is saved until you review the validation screen.</t>
+  </si>
+  <si>
+    <t>UNITS - USE BASE UNITS ONLY</t>
+  </si>
+  <si>
+    <t>Only use g (grams), ml (millilitres), pc (pieces). Convert kg to g and litres to ml - the system does NOT auto-convert.</t>
+  </si>
+  <si>
+    <t>UNIT EXAMPLES</t>
+  </si>
+  <si>
+    <t>1 kg coffee beans  =  1000 g   |   1 litre milk  =  1000 ml   |   1 box of cups  =  the number of pieces, e.g. 500 pc</t>
   </si>
   <si>
     <t>NAMES MUST MATCH</t>
   </si>
   <si>
-    <t>In the Recipes tab, 'Inventory Item Used' must match an Item Name in the Current Stock tab exactly, and 'Menu Item Name' must match a product in the Menu Manager exactly. The importer warns about mismatches before saving.</t>
+    <t>In the Recipes tab, 'Inventory Item Used' and 'Replaces Inventory Item' must match an Item Name in the Current Stock tab exactly, and 'Menu Item' must match a product in the Menu Manager exactly. The importer warns about mismatches before saving.</t>
   </si>
   <si>
     <t>SIZE column</t>
   </si>
   <si>
-    <t>Blank = recipe applies to ALL sizes. Or put Small / Medium / Large to make that line size-specific.</t>
+    <t>Blank = the recipe line applies to ALL sizes. Or put Small / Medium / Large to make that line size-specific.</t>
   </si>
   <si>
     <t>ADD-ON column</t>
@@ -78,46 +87,70 @@
     <t>Blank = base recipe (always deducted). Put an add-on name = only deducted when that add-on is chosen.</t>
   </si>
   <si>
-    <t>DEDUCTION RULE</t>
-  </si>
-  <si>
-    <t>ADD = consume on top of the base recipe (extra shot, syrup, boba). REPLACE = swap out the base ingredient (Oat Milk replaces regular Milk). For REPLACE, model the choice as a single-select add-on group (Milk: Regular / Oat / Almond).</t>
+    <t>DEDUCTION RULE - ADD</t>
+  </si>
+  <si>
+    <t>ADD means the ingredient is added ON TOP of the normal recipe (extra shot, syrup, boba).</t>
+  </si>
+  <si>
+    <t>DEDUCTION RULE - REPLACE</t>
+  </si>
+  <si>
+    <t>REPLACE means this ingredient replaces another one. Put the replaced item in the 'Replaces Inventory Item' column. Example: a regular latte uses Milk; if the customer chooses Oat Milk, oat milk REPLACES milk, so regular milk is NOT deducted (Oat Milk 250 ml, Rule=REPLACE, Replaces=Milk).</t>
+  </si>
+  <si>
+    <t>REPLACES INVENTORY ITEM</t>
+  </si>
+  <si>
+    <t>Only used on REPLACE rows - the base ingredient being swapped out. Leave blank on all normal / ADD rows.</t>
   </si>
   <si>
     <t>DATES</t>
   </si>
   <si>
-    <t>Use format YYYY-MM-DD, e.g. 2026-12-31. Blank if not tracked.</t>
-  </si>
-  <si>
-    <t>HANSON</t>
-  </si>
-  <si>
-    <t>Hanson doughnuts are tracked DAILY on the 'D - Hanson Daily' tab (not the Products tab). Enter how many you made each morning.</t>
+    <t>Use format YYYY-MM-DD, e.g. 2026-12-31. Leave blank if not tracked.</t>
+  </si>
+  <si>
+    <t>STORAGE LOCATION (optional)</t>
+  </si>
+  <si>
+    <t>Where the item is kept. Examples: Fridge, Freezer, Dry Storage, Bar, Kitchen, Display Fridge.</t>
+  </si>
+  <si>
+    <t>BATCH / LOT NUMBER (optional)</t>
+  </si>
+  <si>
+    <t>Reference for a specific delivery batch, for tracing. Leave blank if you do not track batches.</t>
+  </si>
+  <si>
+    <t>HANSON - IMPORTANT</t>
+  </si>
+  <si>
+    <t>Do NOT list daily Hanson doughnuts in the Products tab. Hanson daily stock is entered on the 'D - Hanson Daily' tab, one row per doughnut per day.</t>
   </si>
   <si>
     <t>VALIDATION</t>
   </si>
   <si>
-    <t>Nothing is saved until you review. The importer shows errors like: 'Vanilla Syrup used in a recipe but missing from Current Stock', or 'Unit mismatch: recipe uses ml but item is tracked in g'.</t>
+    <t>The importer shows errors like: 'Vanilla Syrup used in a recipe but missing from Current Stock', 'Iced Latte Medium not found in the menu', or 'Unit mismatch: recipe uses ml but item is tracked in g'. Fix them, then import.</t>
   </si>
   <si>
     <t>Item Name</t>
   </si>
   <si>
-    <t>Inventory Category</t>
+    <t>Category</t>
   </si>
   <si>
     <t>Unit</t>
   </si>
   <si>
-    <t>Current Quantity</t>
-  </si>
-  <si>
-    <t>Minimum Quantity</t>
-  </si>
-  <si>
-    <t>Cost per Unit</t>
+    <t>Current Qty</t>
+  </si>
+  <si>
+    <t>Min Qty</t>
+  </si>
+  <si>
+    <t>Cost/Unit</t>
   </si>
   <si>
     <t>Supplier</t>
@@ -129,6 +162,12 @@
     <t>Track Expiry</t>
   </si>
   <si>
+    <t>Batch / Lot Number</t>
+  </si>
+  <si>
+    <t>Storage Location</t>
+  </si>
+  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -150,6 +189,9 @@
     <t>No</t>
   </si>
   <si>
+    <t>Display Fridge</t>
+  </si>
+  <si>
     <t>Enter ml, not litres</t>
   </si>
   <si>
@@ -171,6 +213,9 @@
     <t>Supplier B</t>
   </si>
   <si>
+    <t>Dry Storage</t>
+  </si>
+  <si>
     <t>Matcha Powder</t>
   </si>
   <si>
@@ -192,6 +237,9 @@
     <t>Supplier D</t>
   </si>
   <si>
+    <t>Bar</t>
+  </si>
+  <si>
     <t>Boba Pearls</t>
   </si>
   <si>
@@ -231,7 +279,10 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Menu Item Name</t>
+    <t>LOT-2026-07</t>
+  </si>
+  <si>
+    <t>Menu Item</t>
   </si>
   <si>
     <t>Menu Category</t>
@@ -240,18 +291,21 @@
     <t>Size</t>
   </si>
   <si>
-    <t>Add-on (if any)</t>
+    <t>Add-on</t>
   </si>
   <si>
     <t>Inventory Item Used</t>
   </si>
   <si>
-    <t>Quantity Used</t>
+    <t>Qty Used</t>
   </si>
   <si>
     <t>Deduction Rule</t>
   </si>
   <si>
+    <t>Replaces Inventory Item</t>
+  </si>
+  <si>
     <t>Iced Latte</t>
   </si>
   <si>
@@ -294,7 +348,7 @@
     <t>REPLACE</t>
   </si>
   <si>
-    <t>replaces regular milk (single-select Milk group)</t>
+    <t>oat milk replaces regular milk</t>
   </si>
   <si>
     <t>Iced Tea</t>
@@ -306,7 +360,10 @@
     <t>Product Name</t>
   </si>
   <si>
-    <t>Product Type</t>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Cost</t>
   </si>
   <si>
     <t>Croissant</t>
@@ -324,6 +381,9 @@
     <t>Brownie</t>
   </si>
   <si>
+    <t>Chocolate Muffin</t>
+  </si>
+  <si>
     <t>Chicken Sandwich</t>
   </si>
   <si>
@@ -348,19 +408,22 @@
     <t>Illy Coffee Machine X1</t>
   </si>
   <si>
+    <t>Illy Beans Bag 250g</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
-    <t>Doughnut Name</t>
-  </si>
-  <si>
-    <t>Hanson Category</t>
-  </si>
-  <si>
-    <t>Quantity Produced</t>
-  </si>
-  <si>
-    <t>Cost per Piece (optional)</t>
+    <t>Doughnut</t>
+  </si>
+  <si>
+    <t>Qty Produced</t>
+  </si>
+  <si>
+    <t>Cost/Piece</t>
+  </si>
+  <si>
+    <t>Available Today</t>
   </si>
   <si>
     <t>2026-07-13</t>
@@ -385,6 +448,9 @@
   </si>
   <si>
     <t>Creation</t>
+  </si>
+  <si>
+    <t>reserved for an order</t>
   </si>
 </sst>
 </file>
@@ -772,90 +838,132 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A677E7-334A-4868-8718-075ED68B9E84}">
-  <dimension ref="A1:B10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CAEB59E-5081-4889-82F6-0C054907C411}">
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="189.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="236.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -864,63 +972,70 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A77E3984-D3D1-421D-BECE-A643FE4C4B1F}">
-  <dimension ref="A1:J12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{195E3611-4A2E-417D-A39B-959A050401AE}">
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D2">
         <v>20000</v>
@@ -932,27 +1047,30 @@
         <v>1.1999999999999999E-3</v>
       </c>
       <c r="G2" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D3">
         <v>8000</v>
@@ -964,24 +1082,27 @@
         <v>2.5000000000000001E-3</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="D4">
         <v>10000</v>
@@ -993,24 +1114,27 @@
         <v>0.02</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="D5">
         <v>1000</v>
@@ -1022,24 +1146,27 @@
         <v>0.08</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="D6">
         <v>2000</v>
@@ -1051,21 +1178,24 @@
         <v>0.05</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D7">
         <v>3000</v>
@@ -1077,24 +1207,27 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="D8">
         <v>2000</v>
@@ -1106,24 +1239,27 @@
         <v>0.01</v>
       </c>
       <c r="G8" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D9">
         <v>500</v>
@@ -1135,24 +1271,27 @@
         <v>0.05</v>
       </c>
       <c r="G9" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D10">
         <v>500</v>
@@ -1164,24 +1303,27 @@
         <v>0.03</v>
       </c>
       <c r="G10" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D11">
         <v>1000</v>
@@ -1193,24 +1335,27 @@
         <v>0.01</v>
       </c>
       <c r="G11" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="K11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D12">
         <v>200</v>
@@ -1222,10 +1367,16 @@
         <v>0.3</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="I12" t="s">
-        <v>61</v>
+        <v>77</v>
+      </c>
+      <c r="J12" t="s">
+        <v>78</v>
+      </c>
+      <c r="K12" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1234,357 +1385,364 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00B4439C-F006-4DF2-8FC0-142C8E492A54}">
-  <dimension ref="A1:I13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF22C1F-A334-4CEB-BBE9-35076CB83E95}">
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="4.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="38.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="F2">
         <v>18</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="H2" t="s">
-        <v>72</v>
-      </c>
-      <c r="I2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+      <c r="J2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F3">
         <v>250</v>
       </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="H4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5" t="s">
-        <v>71</v>
-      </c>
-      <c r="E5" t="s">
-        <v>56</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="H5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="H6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F7">
         <v>180</v>
       </c>
       <c r="G7" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>72</v>
-      </c>
-      <c r="I7" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+      <c r="J7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F8">
         <v>250</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H8" t="s">
-        <v>72</v>
-      </c>
-      <c r="I8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+      <c r="J8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C9" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F9">
         <v>320</v>
       </c>
       <c r="G9" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+      <c r="J9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="D10" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="F10">
         <v>9</v>
       </c>
       <c r="G10" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="H10" t="s">
-        <v>72</v>
-      </c>
-      <c r="I10" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+      <c r="J10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="D11" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="E11" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="F11">
         <v>15</v>
       </c>
       <c r="G11" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H11" t="s">
-        <v>72</v>
-      </c>
-      <c r="I11" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+      <c r="J11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B12" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C12" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="F12">
         <v>250</v>
       </c>
       <c r="G12" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H12" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="I12" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+      <c r="J12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="D13" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="F13">
         <v>40</v>
       </c>
       <c r="G13" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="H13" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1593,15 +1751,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43A515DD-E9A8-44D3-86F6-9439663CF0D1}">
-  <dimension ref="A1:H8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0C2D4C0-DC91-4CD5-816B-BC58019AE6A5}">
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
@@ -1609,36 +1767,36 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>24</v>
+        <v>106</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="C2">
         <v>30</v>
@@ -1650,18 +1808,18 @@
         <v>0.5</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="B3" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -1673,119 +1831,165 @@
         <v>0.6</v>
       </c>
       <c r="F3" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="C4">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4">
-        <v>1.2</v>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="F4" t="s">
+        <v>109</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="H4" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="C5">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>94</v>
+        <v>114</v>
+      </c>
+      <c r="H5" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>116</v>
       </c>
       <c r="B6" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="C6">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>0.3</v>
+        <v>1.5</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="C7">
+        <v>200</v>
+      </c>
+      <c r="D7">
         <v>40</v>
       </c>
-      <c r="D7">
-        <v>10</v>
-      </c>
       <c r="E7">
-        <v>8</v>
-      </c>
-      <c r="F7" t="s">
-        <v>99</v>
+        <v>0.3</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B8" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="C8">
+        <v>40</v>
+      </c>
+      <c r="D8">
+        <v>10</v>
+      </c>
+      <c r="E8">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9">
         <v>5</v>
       </c>
-      <c r="D8">
+      <c r="D9">
         <v>1</v>
       </c>
-      <c r="E8">
+      <c r="E9">
         <v>180</v>
       </c>
-      <c r="F8" t="s">
-        <v>99</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>33</v>
+      <c r="F9" t="s">
+        <v>119</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>121</v>
+      </c>
+      <c r="B10" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10">
+        <v>25</v>
+      </c>
+      <c r="D10">
+        <v>6</v>
+      </c>
+      <c r="E10">
+        <v>6.5</v>
+      </c>
+      <c r="F10" t="s">
+        <v>119</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1794,47 +1998,51 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECDAB600-2DFC-4B1E-804D-AA19C5810A83}">
-  <dimension ref="A1:F5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F361C870-83BB-41E1-A054-DABEA905244D}">
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>103</v>
+        <v>31</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -1842,16 +2050,19 @@
       <c r="E2">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B3" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="D3">
         <v>18</v>
@@ -1859,16 +2070,19 @@
       <c r="E3">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="C4" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="D4">
         <v>8</v>
@@ -1876,22 +2090,31 @@
       <c r="E4">
         <v>1.2</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="B5" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="D5">
         <v>6</v>
       </c>
       <c r="E5">
         <v>1.5</v>
+      </c>
+      <c r="F5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>